<commit_message>
versie 2.0 naar mockup
widgets gekoppeld aan aangepaste code
</commit_message>
<xml_diff>
--- a/import/c_phi_data_geforceerd.xlsx
+++ b/import/c_phi_data_geforceerd.xlsx
@@ -510,37 +510,37 @@
         <v>20.840000152588</v>
       </c>
       <c r="H2">
-        <v>13.17898383273264</v>
+        <v>9.9020746549891</v>
       </c>
       <c r="I2">
-        <v>17.94773050078498</v>
+        <v>21.22463967852851</v>
       </c>
       <c r="J2">
         <v>48425.79727508202</v>
       </c>
       <c r="K2">
-        <v>-2900.149026338879</v>
+        <v>-2179.036907085044</v>
       </c>
       <c r="L2">
-        <v>1.179783012480086</v>
+        <v>0.2298293414006464</v>
       </c>
       <c r="M2">
-        <v>54.56</v>
+        <v>58.5</v>
       </c>
       <c r="N2">
-        <v>5.20612533301011</v>
+        <v>2.749517329212706</v>
       </c>
       <c r="O2">
-        <v>12.70175932396434</v>
+        <v>9.901764788491688</v>
       </c>
       <c r="P2">
-        <v>18.42495500955327</v>
+        <v>21.22432981922115</v>
       </c>
       <c r="Q2">
-        <v>-2795.131658382791</v>
+        <v>-2178.968718290508</v>
       </c>
       <c r="R2">
-        <v>2.444227929496325</v>
+        <v>0.2301265406353878</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -566,37 +566,37 @@
         <v>32.12505770952285</v>
       </c>
       <c r="H3">
-        <v>19.51590318852269</v>
+        <v>16.17567064198671</v>
       </c>
       <c r="I3">
-        <v>24.06879877445653</v>
+        <v>27.40903132099251</v>
       </c>
       <c r="J3">
         <v>43586.4013606754</v>
       </c>
       <c r="K3">
-        <v>-4074.404679023864</v>
+        <v>-3377.052423011561</v>
       </c>
       <c r="L3">
-        <v>0.8385023160065448</v>
+        <v>0.1638346036939383</v>
       </c>
       <c r="M3">
-        <v>102.19</v>
+        <v>106.13</v>
       </c>
       <c r="N3">
-        <v>37.82660943187111</v>
+        <v>4.886753265765213</v>
       </c>
       <c r="O3">
-        <v>19.06027962310524</v>
+        <v>16.17537607564727</v>
       </c>
       <c r="P3">
-        <v>24.52442233987398</v>
+        <v>27.40873676178646</v>
       </c>
       <c r="Q3">
-        <v>-3979.282523063275</v>
+        <v>-3376.990925346805</v>
       </c>
       <c r="R3">
-        <v>1.880522070225117</v>
+        <v>0.1640731506781457</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -622,37 +622,37 @@
         <v>43.41011526645769</v>
       </c>
       <c r="H4">
-        <v>25.84775021722176</v>
+        <v>22.44555813639322</v>
       </c>
       <c r="I4">
-        <v>30.19493937521905</v>
+        <v>33.59713145604758</v>
       </c>
       <c r="J4">
         <v>39001.71049439544</v>
       </c>
       <c r="K4">
-        <v>-5104.633606075894</v>
+        <v>-4432.739770667679</v>
       </c>
       <c r="L4">
-        <v>0.5629344852255217</v>
+        <v>0.1114445028195387</v>
       </c>
       <c r="M4">
-        <v>50.31</v>
+        <v>54.25</v>
       </c>
       <c r="N4">
-        <v>3.612583131401773</v>
+        <v>4.1583044463321</v>
       </c>
       <c r="O4">
-        <v>25.41271238551085</v>
+        <v>22.44527887020941</v>
       </c>
       <c r="P4">
-        <v>30.62997720692995</v>
+        <v>33.59685219694523</v>
       </c>
       <c r="Q4">
-        <v>-5018.718634095613</v>
+        <v>-4432.684618805913</v>
       </c>
       <c r="R4">
-        <v>1.405001122510772</v>
+        <v>0.111631037370897</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -678,37 +678,37 @@
         <v>54.69517282339254</v>
       </c>
       <c r="H5">
-        <v>32.17377107887813</v>
+        <v>28.71165499502634</v>
       </c>
       <c r="I5">
-        <v>36.32690614302428</v>
+        <v>39.78902222687607</v>
       </c>
       <c r="J5">
         <v>34671.72467624215</v>
       </c>
       <c r="K5">
-        <v>-5990.867164404954</v>
+        <v>-5346.209206366509</v>
       </c>
       <c r="L5">
-        <v>0.3489355253842005</v>
+        <v>0.07112454490776596</v>
       </c>
       <c r="M5">
-        <v>14.88</v>
+        <v>18.82</v>
       </c>
       <c r="N5">
-        <v>23.28320753568169</v>
+        <v>0.7837844454196563</v>
       </c>
       <c r="O5">
-        <v>31.7581528926336</v>
+        <v>28.71139102899574</v>
       </c>
       <c r="P5">
-        <v>36.7425243292688</v>
+        <v>39.78875826787981</v>
       </c>
       <c r="Q5">
-        <v>-5913.477624372561</v>
+        <v>-5346.160054981011</v>
       </c>
       <c r="R5">
-        <v>1.012691684631328</v>
+        <v>0.07126540976593447</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -734,37 +734,37 @@
         <v>65.98023038032738</v>
       </c>
       <c r="H6">
-        <v>38.49311176363879</v>
+        <v>34.9738845782874</v>
       </c>
       <c r="I6">
-        <v>42.46555308772521</v>
+        <v>45.9847802730766</v>
       </c>
       <c r="J6">
         <v>30596.44390621552</v>
       </c>
       <c r="K6">
-        <v>-6733.153217871932</v>
+        <v>-6117.575657061318</v>
       </c>
       <c r="L6">
-        <v>0.1916739815180599</v>
+        <v>0.04137885698653937</v>
       </c>
       <c r="M6">
-        <v>45.42</v>
+        <v>49.36</v>
       </c>
       <c r="N6">
-        <v>21.61359822754606</v>
+        <v>0.5029159971931801</v>
       </c>
       <c r="O6">
-        <v>38.09557620734718</v>
+        <v>34.97363591240757</v>
       </c>
       <c r="P6">
-        <v>42.86308864401683</v>
+        <v>45.98453161418889</v>
       </c>
       <c r="Q6">
-        <v>-6663.616937549908</v>
+        <v>-6117.532160825439</v>
       </c>
       <c r="R6">
-        <v>0.6977953017446787</v>
+        <v>0.04148008502168629</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -790,37 +790,37 @@
         <v>77.26528793726223</v>
       </c>
       <c r="H7">
-        <v>44.80482084166709</v>
+        <v>41.23217647208939</v>
       </c>
       <c r="I7">
-        <v>48.61183163915852</v>
+        <v>52.18447600873621</v>
       </c>
       <c r="J7">
         <v>26775.86818431555</v>
       </c>
       <c r="K7">
-        <v>-7331.562239382315</v>
+        <v>-6746.958527935734</v>
       </c>
       <c r="L7">
-        <v>0.08557713733081966</v>
+        <v>0.02075953889376583</v>
       </c>
       <c r="M7">
-        <v>92.26000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="N7">
-        <v>9.597852674180466</v>
+        <v>0.7085020529279198</v>
       </c>
       <c r="O7">
-        <v>44.42384047425108</v>
+        <v>41.23194310635781</v>
       </c>
       <c r="P7">
-        <v>48.99281200657452</v>
+        <v>52.18424264995955</v>
       </c>
       <c r="Q7">
-        <v>-7269.221151454213</v>
+        <v>-6746.9203415229</v>
       </c>
       <c r="R7">
-        <v>0.4536238966507215</v>
+        <v>0.02082684082022829</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -846,37 +846,37 @@
         <v>88.55034549419707</v>
       </c>
       <c r="H8">
-        <v>51.10786287624045</v>
+        <v>47.48646718137286</v>
       </c>
       <c r="I8">
-        <v>54.76677723404675</v>
+        <v>58.38817292891434</v>
       </c>
       <c r="J8">
         <v>23209.99751054226</v>
       </c>
       <c r="K8">
-        <v>-7786.194851299138</v>
+        <v>-7234.481456783412</v>
       </c>
       <c r="L8">
-        <v>0.02431496851382262</v>
+        <v>0.007875970718547069</v>
       </c>
       <c r="M8">
-        <v>43.57</v>
+        <v>47.51</v>
       </c>
       <c r="N8">
-        <v>0.0361172068666924</v>
+        <v>14.06135430388009</v>
       </c>
       <c r="O8">
-        <v>50.74170301735608</v>
+        <v>47.48624911578699</v>
       </c>
       <c r="P8">
-        <v>55.13293709293112</v>
+        <v>58.38795487025126</v>
       </c>
       <c r="Q8">
-        <v>-7730.411027684723</v>
+        <v>-7234.448234867127</v>
       </c>
       <c r="R8">
-        <v>0.2725805114200511</v>
+        <v>0.007914723458558712</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -902,37 +902,37 @@
         <v>99.83540305113192</v>
       </c>
       <c r="H9">
-        <v>57.40114679067597</v>
+        <v>53.73670078057049</v>
       </c>
       <c r="I9">
-        <v>60.93148094907284</v>
+        <v>64.59592695917831</v>
       </c>
       <c r="J9">
         <v>19898.83188489562</v>
       </c>
       <c r="K9">
-        <v>-8097.190567085543</v>
+        <v>-7580.272015356536</v>
       </c>
       <c r="L9">
-        <v>0.0008460867935685585</v>
+        <v>0.001403905946059814</v>
       </c>
       <c r="M9">
-        <v>59.56</v>
+        <v>63.5</v>
       </c>
       <c r="N9">
-        <v>0.07762168062996844</v>
+        <v>17.79541376375152</v>
       </c>
       <c r="O9">
-        <v>57.04785438455682</v>
+        <v>53.73649801512776</v>
       </c>
       <c r="P9">
-        <v>61.28477335519198</v>
+        <v>64.59572420063139</v>
       </c>
       <c r="Q9">
-        <v>-8047.354002867011</v>
+        <v>-7580.243412610389</v>
       </c>
       <c r="R9">
-        <v>0.1462144469921932</v>
+        <v>0.001419141788319563</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -958,37 +958,37 @@
         <v>111.1204606080668</v>
       </c>
       <c r="H10">
-        <v>63.68357273222762</v>
+        <v>59.9828295064279</v>
       </c>
       <c r="I10">
-        <v>67.10704263698277</v>
+        <v>70.80778586278251</v>
       </c>
       <c r="J10">
         <v>16842.37130737565</v>
       </c>
       <c r="K10">
-        <v>-8264.737012715994</v>
+        <v>-7784.461359190249</v>
       </c>
       <c r="L10">
-        <v>0.00755151644368676</v>
+        <v>9.417395849304534E-05</v>
       </c>
       <c r="M10">
-        <v>116.9</v>
+        <v>120.84</v>
       </c>
       <c r="N10">
-        <v>27.42425083020706</v>
+        <v>84.20893381163276</v>
       </c>
       <c r="O10">
-        <v>63.34097459118461</v>
+        <v>59.9826420411257</v>
       </c>
       <c r="P10">
-        <v>67.4496407780258</v>
+        <v>70.80759840435437</v>
       </c>
       <c r="Q10">
-        <v>-8220.275255699447</v>
+        <v>-7784.437030287909</v>
       </c>
       <c r="R10">
-        <v>0.06538181461794615</v>
+        <v>9.05706526230713E-05</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -1014,37 +1014,37 @@
         <v>122.4055181650016</v>
       </c>
       <c r="H11">
-        <v>69.95409829057496</v>
+        <v>66.22481427918164</v>
       </c>
       <c r="I11">
-        <v>73.29450470809701</v>
+        <v>77.02378871949033</v>
       </c>
       <c r="J11">
         <v>14040.61577798234</v>
       </c>
       <c r="K11">
-        <v>-8289.078268302455</v>
+        <v>-7847.183828797787</v>
       </c>
       <c r="L11">
-        <v>0.03647569471460082</v>
+        <v>0.002780814997462076</v>
       </c>
       <c r="M11">
-        <v>27.63</v>
+        <v>31.57</v>
       </c>
       <c r="N11">
-        <v>20.85118518904353</v>
+        <v>0.3923630327124475</v>
       </c>
       <c r="O11">
-        <v>69.61981259190951</v>
+        <v>66.22464211401736</v>
       </c>
       <c r="P11">
-        <v>73.62879040676246</v>
+        <v>77.0236165611836</v>
       </c>
       <c r="Q11">
-        <v>-8249.467718128508</v>
+        <v>-7847.16342841301</v>
       </c>
       <c r="R11">
-        <v>0.02053477173527912</v>
+        <v>0.002762686917858693</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -1070,37 +1070,37 @@
         <v>133.6905757219365</v>
       </c>
       <c r="H12">
-        <v>76.21181992540581</v>
+        <v>72.46262513925232</v>
       </c>
       <c r="I12">
-        <v>79.49477070272776</v>
+        <v>83.24396548888124</v>
       </c>
       <c r="J12">
         <v>11493.5652967157</v>
       </c>
       <c r="K12">
-        <v>-8170.520356581093</v>
+        <v>-7768.576506519023</v>
       </c>
       <c r="L12">
-        <v>0.07967569657313057</v>
+        <v>0.008388476652801321</v>
       </c>
       <c r="M12">
-        <v>163.5</v>
+        <v>167.44</v>
       </c>
       <c r="N12">
-        <v>81.81717124453857</v>
+        <v>26.06825718839467</v>
       </c>
       <c r="O12">
-        <v>75.88328400578695</v>
+        <v>72.4624682742233</v>
       </c>
       <c r="P12">
-        <v>79.82330662234662</v>
+        <v>83.24380863069858</v>
       </c>
       <c r="Q12">
-        <v>-8135.298662338109</v>
+        <v>-7768.559689325652</v>
       </c>
       <c r="R12">
-        <v>0.002140642896065892</v>
+        <v>0.008359767154075194</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -1126,37 +1126,37 @@
         <v>144.9756332788713</v>
       </c>
       <c r="H13">
-        <v>82.4560589402132</v>
+        <v>78.69624158831694</v>
       </c>
       <c r="I13">
-        <v>85.70851931738197</v>
+        <v>89.46833666927823</v>
       </c>
       <c r="J13">
         <v>9201.219863575725</v>
       </c>
       <c r="K13">
-        <v>-7909.43165399569</v>
+        <v>-7548.778734628141</v>
       </c>
       <c r="L13">
-        <v>0.1296496440619567</v>
+        <v>0.0159389135817621</v>
       </c>
       <c r="M13">
-        <v>58.86</v>
+        <v>62.8</v>
       </c>
       <c r="N13">
-        <v>133.8915722205397</v>
+        <v>58.23713020895935</v>
       </c>
       <c r="O13">
-        <v>82.1305742974283</v>
+        <v>78.6961000234205</v>
       </c>
       <c r="P13">
-        <v>86.03400396016687</v>
+        <v>89.46819511122227</v>
       </c>
       <c r="Q13">
-        <v>-7878.210194110019</v>
+        <v>-7548.765155300104</v>
       </c>
       <c r="R13">
-        <v>0.001196073854871941</v>
+        <v>0.01590318865301467</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -1182,37 +1182,37 @@
         <v>156.2606908358061</v>
       </c>
       <c r="H14">
-        <v>88.68643578683758</v>
+        <v>84.92565282582993</v>
       </c>
       <c r="I14">
-        <v>91.93613010021919</v>
+        <v>95.69691306122684</v>
       </c>
       <c r="J14">
         <v>7163.579478562413</v>
       </c>
       <c r="K14">
-        <v>-7506.236492803998</v>
+        <v>-7187.931601498165</v>
       </c>
       <c r="L14">
-        <v>0.1797818354534798</v>
+        <v>0.02455645125316587</v>
       </c>
       <c r="M14">
-        <v>50.73</v>
+        <v>54.66999999999999</v>
       </c>
       <c r="N14">
-        <v>24.63731999284618</v>
+        <v>1.048036008883847</v>
       </c>
       <c r="O14">
-        <v>88.36122795335372</v>
+        <v>84.92552656106342</v>
       </c>
       <c r="P14">
-        <v>92.26133793370305</v>
+        <v>95.69678680330027</v>
       </c>
       <c r="Q14">
-        <v>-7478.711574412762</v>
+        <v>-7187.920914709484</v>
       </c>
       <c r="R14">
-        <v>0.009761251864225528</v>
+        <v>0.02451689456013674</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1238,37 +1238,37 @@
         <v>167.545748392741</v>
       </c>
       <c r="H15">
-        <v>94.90291533798306</v>
+        <v>91.15085787468156</v>
       </c>
       <c r="I15">
-        <v>98.1776381785353</v>
+        <v>101.9296956418368</v>
       </c>
       <c r="J15">
         <v>5380.644141675764</v>
       </c>
       <c r="K15">
-        <v>-6961.401602415333</v>
+        <v>-6686.177403618485</v>
       </c>
       <c r="L15">
-        <v>0.2247210548086066</v>
+        <v>0.03347229941010008</v>
       </c>
       <c r="M15">
-        <v>8.920000000000002</v>
+        <v>12.86</v>
       </c>
       <c r="N15">
-        <v>23.43111049144251</v>
+        <v>0.8110858211229168</v>
       </c>
       <c r="O15">
-        <v>94.57520281565418</v>
+        <v>91.15074691004229</v>
       </c>
       <c r="P15">
-        <v>98.50535070086418</v>
+        <v>101.9295846840423</v>
       </c>
       <c r="Q15">
-        <v>-6937.36294701737</v>
+        <v>-6686.169264043269</v>
       </c>
       <c r="R15">
-        <v>0.02141393265175408</v>
+        <v>0.03343170879317794</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -1294,37 +1294,37 @@
         <v>178.8308059496758</v>
       </c>
       <c r="H16">
-        <v>101.1058112136215</v>
+        <v>97.37186559260125</v>
       </c>
       <c r="I16">
-        <v>104.4327299323584</v>
+        <v>108.1666755533787</v>
       </c>
       <c r="J16">
         <v>3852.413852915781</v>
       </c>
       <c r="K16">
-        <v>-6275.416943874675</v>
+        <v>-6043.659092012444</v>
       </c>
       <c r="L16">
-        <v>0.2606148350165677</v>
+        <v>0.0420276306215713</v>
       </c>
       <c r="M16">
-        <v>41.13</v>
+        <v>45.07</v>
       </c>
       <c r="N16">
-        <v>3.959818347247407</v>
+        <v>35.1629205095526</v>
       </c>
       <c r="O16">
-        <v>100.7728752743111</v>
+        <v>97.37176992808656</v>
       </c>
       <c r="P16">
-        <v>104.7656658716688</v>
+        <v>108.1665798957189</v>
       </c>
       <c r="Q16">
-        <v>-6254.75233706628</v>
+        <v>-6043.653154324894</v>
       </c>
       <c r="R16">
-        <v>0.03153059043971856</v>
+        <v>0.04198841609467178</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -1350,37 +1350,37 @@
         <v>190.1158635066107</v>
       </c>
       <c r="H17">
-        <v>107.2957479732355</v>
+        <v>103.5886945689971</v>
       </c>
       <c r="I17">
-        <v>110.7007808022061</v>
+        <v>114.4078342064445</v>
       </c>
       <c r="J17">
         <v>2578.888612282462</v>
       </c>
       <c r="K17">
-        <v>-5448.774111715502</v>
+        <v>-5260.519712064926</v>
       </c>
       <c r="L17">
-        <v>0.2851585008045973</v>
+        <v>0.04967537239241795</v>
       </c>
       <c r="M17">
-        <v>201.050003051758</v>
+        <v>204.990003051758</v>
       </c>
       <c r="N17">
-        <v>608.5371501485484</v>
+        <v>818.4241021391014</v>
       </c>
       <c r="O17">
-        <v>106.9549948923407</v>
+        <v>103.5886142046043</v>
       </c>
       <c r="P17">
-        <v>111.0415338831008</v>
+        <v>114.4077538489221</v>
       </c>
       <c r="Q17">
-        <v>-5431.469730127802</v>
+        <v>-5260.515630939335</v>
       </c>
       <c r="R17">
-        <v>0.03734527675238551</v>
+        <v>0.04963955566312393</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -1406,37 +1406,37 @@
         <v>201.4009210635455</v>
       </c>
       <c r="H18">
-        <v>113.4735912658377</v>
+        <v>109.8013729100198</v>
       </c>
       <c r="I18">
-        <v>116.9809251390655</v>
+        <v>120.6531434948833</v>
       </c>
       <c r="J18">
         <v>1560.068419775808</v>
       </c>
       <c r="K18">
-        <v>-4481.946030194753</v>
+        <v>-4336.901845920123</v>
       </c>
       <c r="L18">
-        <v>0.2974684961560704</v>
+        <v>0.05598069623610943</v>
       </c>
       <c r="M18">
-        <v>43.990001678467</v>
+        <v>47.930001678467</v>
       </c>
       <c r="N18">
-        <v>18.03281333628908</v>
+        <v>0.09401858233828998</v>
       </c>
       <c r="O18">
-        <v>113.1226005755687</v>
+        <v>109.8013078457464</v>
       </c>
       <c r="P18">
-        <v>117.3319158293344</v>
+        <v>120.6530784375009</v>
       </c>
       <c r="Q18">
-        <v>-4468.082704699036</v>
+        <v>-4336.899276030875</v>
       </c>
       <c r="R18">
-        <v>0.03779759473194401</v>
+        <v>0.05594991174280269</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -1462,37 +1462,37 @@
         <v>212.6859786204804</v>
       </c>
       <c r="H19">
-        <v>119.6403627614145</v>
+        <v>116.0099379176039</v>
       </c>
       <c r="I19">
-        <v>123.2721412729502</v>
+        <v>126.9025661167609</v>
       </c>
       <c r="J19">
         <v>795.9532753958177</v>
       </c>
       <c r="K19">
-        <v>-3375.370949737799</v>
+        <v>-3272.947066441477</v>
       </c>
       <c r="L19">
-        <v>0.2978313969722741</v>
+        <v>0.06062022219138373</v>
       </c>
       <c r="M19">
-        <v>19.079999923706</v>
+        <v>23.019999923706</v>
       </c>
       <c r="N19">
-        <v>17.19616860493785</v>
+        <v>0.04280073323022309</v>
       </c>
       <c r="O19">
-        <v>119.2769184778811</v>
+        <v>116.0098881534471</v>
       </c>
       <c r="P19">
-        <v>123.6355855564837</v>
+        <v>126.9025163595211</v>
       </c>
       <c r="Q19">
-        <v>-3365.117225591765</v>
+        <v>-3272.945662463042</v>
       </c>
       <c r="R19">
-        <v>0.03323147750718273</v>
+        <v>0.06059571962832663</v>
       </c>
     </row>
     <row r="20" spans="1:18">
@@ -1518,37 +1518,37 @@
         <v>223.9710361774152</v>
       </c>
       <c r="H20">
-        <v>125.7971567621093</v>
+        <v>122.2144356709254</v>
       </c>
       <c r="I20">
-        <v>129.573334901717</v>
+        <v>133.156055992901</v>
       </c>
       <c r="J20">
         <v>286.5431791424922</v>
       </c>
       <c r="K20">
-        <v>-2129.442231838719</v>
+        <v>-2068.795411252037</v>
       </c>
       <c r="L20">
-        <v>0.287397210263021</v>
+        <v>0.06337999080047554</v>
       </c>
       <c r="M20">
-        <v>31.830001831055</v>
+        <v>35.770001831055</v>
       </c>
       <c r="N20">
-        <v>17.8936355442914</v>
+        <v>0.08420183032746099</v>
       </c>
       <c r="O20">
-        <v>125.4192619224088</v>
+        <v>122.2144012068827</v>
       </c>
       <c r="P20">
-        <v>129.9512297414175</v>
+        <v>133.1560215358064</v>
       </c>
       <c r="Q20">
-        <v>-2123.045384313986</v>
+        <v>-2068.794827858979</v>
       </c>
       <c r="R20">
-        <v>0.02502710222213793</v>
+        <v>0.06336263907876868</v>
       </c>
     </row>
     <row r="21" spans="1:18">
@@ -1574,37 +1574,37 @@
         <v>235.2560937343501</v>
       </c>
       <c r="H21">
-        <v>131.9450704402343</v>
+        <v>128.4149205210134</v>
       </c>
       <c r="I21">
-        <v>135.8834088530537</v>
+        <v>139.4135587722746</v>
       </c>
       <c r="J21">
         <v>31.8381310158313</v>
       </c>
       <c r="K21">
-        <v>-744.5038571359127</v>
+        <v>-724.5848846244047</v>
       </c>
       <c r="L21">
-        <v>0.2678778494988603</v>
+        <v>0.06415228502825564</v>
       </c>
       <c r="M21">
-        <v>131.483856201172</v>
+        <v>135.423856201172</v>
       </c>
       <c r="N21">
-        <v>47.41257754745181</v>
+        <v>8.679028170216601</v>
       </c>
       <c r="O21">
-        <v>131.5509476769069</v>
+        <v>128.4149013570822</v>
       </c>
       <c r="P21">
-        <v>136.277531616381</v>
+        <v>139.4135396153278</v>
       </c>
       <c r="Q21">
-        <v>-742.2800081015889</v>
+        <v>-724.5847764913717</v>
       </c>
       <c r="R21">
-        <v>0.01523901621823073</v>
+        <v>0.06414257759904375</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -1630,37 +1630,37 @@
         <v>246.5411512912849</v>
       </c>
       <c r="H22">
-        <v>138.0851530758964</v>
+        <v>134.61145451106</v>
       </c>
       <c r="I22">
-        <v>142.2013138468531</v>
+        <v>145.6750124116895</v>
       </c>
       <c r="J22">
         <v>31.83813101583483</v>
       </c>
       <c r="K22">
-        <v>779.1494501098464</v>
+        <v>759.5490059900357</v>
       </c>
       <c r="L22">
-        <v>0.2412901136815812</v>
+        <v>0.06293141069874647</v>
       </c>
       <c r="M22">
-        <v>242.057250976563</v>
+        <v>245.997250976563</v>
       </c>
       <c r="N22">
-        <v>153.1784167995084</v>
+        <v>71.18553061184967</v>
       </c>
       <c r="O22">
-        <v>137.673235031457</v>
+        <v>134.6114506472379</v>
       </c>
       <c r="P22">
-        <v>142.6132318912925</v>
+        <v>145.675008554893</v>
       </c>
       <c r="Q22">
-        <v>776.8251906897268</v>
+        <v>759.5489841883083</v>
       </c>
       <c r="R22">
-        <v>0.006287674207990829</v>
+        <v>0.06292947214652157</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -1686,37 +1686,37 @@
         <v>257.8262088482197</v>
       </c>
       <c r="H23">
-        <v>144.2183742485364</v>
+        <v>140.8041067362444</v>
       </c>
       <c r="I23">
-        <v>148.5260803036747</v>
+        <v>151.9403478159667</v>
       </c>
       <c r="J23">
         <v>286.5431791425019</v>
       </c>
       <c r="K23">
-        <v>2441.268981243473</v>
+        <v>2383.473673156991</v>
       </c>
       <c r="L23">
-        <v>0.2097595706792486</v>
+        <v>0.0598085648013368</v>
       </c>
       <c r="M23">
-        <v>36.909999847412</v>
+        <v>40.849999847412</v>
       </c>
       <c r="N23">
-        <v>26.57920398623899</v>
+        <v>1.477697039238471</v>
       </c>
       <c r="O23">
-        <v>143.7872876236473</v>
+        <v>140.8041181725289</v>
       </c>
       <c r="P23">
-        <v>148.9571669285638</v>
+        <v>151.9403592593229</v>
       </c>
       <c r="Q23">
-        <v>2433.971725182626</v>
+        <v>2383.473866745684</v>
       </c>
       <c r="R23">
-        <v>0.0007240695024572424</v>
+        <v>0.05981415859947429</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -1742,37 +1742,37 @@
         <v>269.1112664051545</v>
       </c>
       <c r="H24">
-        <v>150.3456077956754</v>
+        <v>146.9929526575888</v>
       </c>
       <c r="I24">
-        <v>154.8568343859972</v>
+        <v>158.2094895240839</v>
       </c>
       <c r="J24">
         <v>795.9532753958322</v>
       </c>
       <c r="K24">
-        <v>4241.647093516389</v>
+        <v>4147.059828011735</v>
       </c>
       <c r="L24">
-        <v>0.1753848989937095</v>
+        <v>0.05496593588997659</v>
       </c>
       <c r="M24">
-        <v>10.590000152588</v>
+        <v>14.530000152588</v>
       </c>
       <c r="N24">
-        <v>21.51850987845511</v>
+        <v>0.4883804149310934</v>
       </c>
       <c r="O24">
-        <v>149.8941541867153</v>
+        <v>146.9929793939774</v>
       </c>
       <c r="P24">
-        <v>155.3082879949573</v>
+        <v>158.2095162675952</v>
       </c>
       <c r="Q24">
-        <v>4228.910393612887</v>
+        <v>4147.060582315947</v>
       </c>
       <c r="R24">
-        <v>0.001066924227839477</v>
+        <v>0.05497847319861389</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -1798,37 +1798,37 @@
         <v>280.3963239620894</v>
       </c>
       <c r="H25">
-        <v>156.4676272792761</v>
+        <v>153.1780733845188</v>
       </c>
       <c r="I25">
-        <v>161.1928025318582</v>
+        <v>164.4823564266154</v>
       </c>
       <c r="J25">
         <v>1560.068419775826</v>
       </c>
       <c r="K25">
-        <v>6180.111628752818</v>
+        <v>6050.181811116407</v>
       </c>
       <c r="L25">
-        <v>0.1401531797321536</v>
+        <v>0.04867018957082105</v>
       </c>
       <c r="M25">
-        <v>123.449996948242</v>
+        <v>127.389996948242</v>
       </c>
       <c r="N25">
-        <v>107.6346276646026</v>
+        <v>41.40973566020971</v>
       </c>
       <c r="O25">
-        <v>155.9947631085151</v>
+        <v>153.1781154210093</v>
       </c>
       <c r="P25">
-        <v>161.6656667026191</v>
+        <v>164.4823984702843</v>
       </c>
       <c r="Q25">
-        <v>6161.434580910044</v>
+        <v>6050.183471461156</v>
       </c>
       <c r="R25">
-        <v>0.009701027262872666</v>
+        <v>0.04868873894829245</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -1854,37 +1854,37 @@
         <v>291.6813815190242</v>
       </c>
       <c r="H26">
-        <v>162.5851089389309</v>
+        <v>159.359554940443</v>
       </c>
       <c r="I26">
-        <v>167.5333085016649</v>
+        <v>170.7588625001528</v>
       </c>
       <c r="J26">
         <v>2578.888612282482</v>
       </c>
       <c r="K26">
-        <v>8256.520405243615</v>
+        <v>8092.717873876894</v>
       </c>
       <c r="L26">
-        <v>0.1058937043076859</v>
+        <v>0.04126549490965226</v>
       </c>
       <c r="M26">
-        <v>10.979999542236</v>
+        <v>14.919999542236</v>
       </c>
       <c r="N26">
-        <v>31.00272704871483</v>
+        <v>2.650546477312232</v>
       </c>
       <c r="O26">
-        <v>162.0899259757777</v>
+        <v>159.3596122770329</v>
       </c>
       <c r="P26">
-        <v>168.0284914648181</v>
+        <v>170.7589198439815</v>
       </c>
       <c r="Q26">
-        <v>8231.373648161825</v>
+        <v>8092.720785587121</v>
       </c>
       <c r="R26">
-        <v>0.02882179670208083</v>
+        <v>0.04128879280394272</v>
       </c>
     </row>
     <row r="27" spans="1:18">
@@ -1910,37 +1910,37 @@
         <v>302.966439075959</v>
       </c>
       <c r="H27">
-        <v>168.6986389335552</v>
+        <v>165.5374875248642</v>
       </c>
       <c r="I27">
-        <v>173.8777661365021</v>
+        <v>177.0389175451931</v>
       </c>
       <c r="J27">
         <v>3852.413852915803</v>
       </c>
       <c r="K27">
-        <v>10470.75617577957</v>
+        <v>10274.55041001663</v>
       </c>
       <c r="L27">
-        <v>0.0742585469507482</v>
+        <v>0.03316624497142829</v>
       </c>
       <c r="M27">
-        <v>35.64</v>
+        <v>39.58</v>
       </c>
       <c r="N27">
-        <v>3.259931890447133</v>
+        <v>4.555577455953099</v>
       </c>
       <c r="O27">
-        <v>168.1803462652042</v>
+        <v>165.5375601615514</v>
       </c>
       <c r="P27">
-        <v>174.3960588048532</v>
+        <v>177.0389901891839</v>
       </c>
       <c r="Q27">
-        <v>10438.58688151434</v>
+        <v>10274.5549184172</v>
       </c>
       <c r="R27">
-        <v>0.06041196401897916</v>
+        <v>0.03319270685633794</v>
       </c>
     </row>
     <row r="28" spans="1:18">
@@ -1966,37 +1966,37 @@
         <v>314.2514966328938</v>
       </c>
       <c r="H28">
-        <v>174.8087226013817</v>
+        <v>171.7119647843776</v>
       </c>
       <c r="I28">
-        <v>180.2256700981373</v>
+        <v>183.3224279151414</v>
       </c>
       <c r="J28">
         <v>5380.644141675785</v>
       </c>
       <c r="K28">
-        <v>12822.72222407052</v>
+        <v>12595.56613773945</v>
       </c>
       <c r="L28">
-        <v>0.04672037880942322</v>
+        <v>0.0248496173458238</v>
       </c>
       <c r="M28">
-        <v>11.78</v>
+        <v>15.72</v>
       </c>
       <c r="N28">
-        <v>33.57820099107776</v>
+        <v>3.439961122799935</v>
       </c>
       <c r="O28">
-        <v>174.2666304568185</v>
+        <v>171.7120527211598</v>
       </c>
       <c r="P28">
-        <v>180.7677622427004</v>
+        <v>183.3225158592964</v>
       </c>
       <c r="Q28">
-        <v>12782.95820722889</v>
+        <v>12595.57258815517</v>
       </c>
       <c r="R28">
-        <v>0.106238950665715</v>
+        <v>0.02487734936774722</v>
       </c>
     </row>
     <row r="29" spans="1:18">
@@ -2022,37 +2022,37 @@
         <v>325.5365541898286</v>
       </c>
       <c r="H29">
-        <v>180.9157942687035</v>
+        <v>177.8830831034738</v>
       </c>
       <c r="I29">
-        <v>186.576586060277</v>
+        <v>189.6092972255067</v>
       </c>
       <c r="J29">
         <v>7163.579478562432</v>
       </c>
       <c r="K29">
-        <v>15312.33863460676</v>
+        <v>15055.65623420794</v>
       </c>
       <c r="L29">
-        <v>0.02458051156323227</v>
+        <v>0.01684810929715163</v>
       </c>
       <c r="M29">
-        <v>19.63</v>
+        <v>23.57</v>
       </c>
       <c r="N29">
-        <v>4.649146821735417</v>
+        <v>3.181794232444192</v>
       </c>
       <c r="O29">
-        <v>180.3492998058981</v>
+        <v>177.8831863403489</v>
       </c>
       <c r="P29">
-        <v>187.1430805230824</v>
+        <v>189.6094004698281</v>
       </c>
       <c r="Q29">
-        <v>15264.39171496843</v>
+        <v>15055.66497196352</v>
       </c>
       <c r="R29">
-        <v>0.1678645215898153</v>
+        <v>0.0168749203028823</v>
       </c>
     </row>
     <row r="30" spans="1:18">
@@ -2078,37 +2078,37 @@
         <v>336.8216117467634</v>
       </c>
       <c r="H30">
-        <v>187.0202267392967</v>
+        <v>184.0509409244641</v>
       </c>
       <c r="I30">
-        <v>192.9301412191454</v>
+        <v>195.899427033978</v>
       </c>
       <c r="J30">
         <v>9201.219863575741</v>
       </c>
       <c r="K30">
-        <v>17939.53919604372</v>
+        <v>17654.71642479502</v>
       </c>
       <c r="L30">
-        <v>0.008982356371106412</v>
+        <v>0.009742168064365382</v>
       </c>
       <c r="M30">
-        <v>17.38</v>
+        <v>21.32</v>
       </c>
       <c r="N30">
-        <v>7.90171931155601</v>
+        <v>1.274529695798266</v>
       </c>
       <c r="O30">
-        <v>186.428801731673</v>
+        <v>184.05105946143</v>
       </c>
       <c r="P30">
-        <v>193.521566226769</v>
+        <v>195.8995455784679</v>
       </c>
       <c r="Q30">
-        <v>17882.80794140475</v>
+        <v>17654.72779521513</v>
       </c>
       <c r="R30">
-        <v>0.2466609379464854</v>
+        <v>0.00976558188658334</v>
       </c>
     </row>
     <row r="31" spans="1:18">
@@ -2134,37 +2134,37 @@
         <v>348.1066693036983</v>
       </c>
       <c r="H31">
-        <v>193.1223400087439</v>
+        <v>190.2156381041452</v>
       </c>
       <c r="I31">
-        <v>199.2860155791597</v>
+        <v>202.1927174837585</v>
       </c>
       <c r="J31">
         <v>11493.56529671571</v>
       </c>
       <c r="K31">
-        <v>20704.26886402184</v>
+        <v>20392.64703022647</v>
       </c>
       <c r="L31">
-        <v>0.0009271814780645421</v>
+        <v>0.004153020797467776</v>
       </c>
       <c r="M31">
-        <v>36.76</v>
+        <v>40.7</v>
       </c>
       <c r="N31">
-        <v>85.29477078004213</v>
+        <v>28.04369486682699</v>
       </c>
       <c r="O31">
-        <v>192.505520275793</v>
+        <v>190.2157719411999</v>
       </c>
       <c r="P31">
-        <v>199.9028353121107</v>
+        <v>202.1928513284189</v>
       </c>
       <c r="Q31">
-        <v>20638.14082523009</v>
+        <v>20392.66137863569</v>
       </c>
       <c r="R31">
-        <v>0.3438298685387012</v>
+        <v>0.004170288682814313</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -2190,37 +2190,37 @@
         <v>359.3917268606331</v>
       </c>
       <c r="H32">
-        <v>199.2224090107087</v>
+        <v>196.3772753131205</v>
       </c>
       <c r="I32">
-        <v>205.6439342066566</v>
+        <v>208.4890679042447</v>
       </c>
       <c r="J32">
         <v>14040.61577798235</v>
       </c>
       <c r="K32">
-        <v>23606.48169932913</v>
+        <v>23269.35297521733</v>
       </c>
       <c r="L32">
-        <v>0.00129026450076935</v>
+        <v>0.0007357915636016385</v>
       </c>
       <c r="M32">
-        <v>210.779998779297</v>
+        <v>214.719998779297</v>
       </c>
       <c r="N32">
-        <v>0.5068272513700383</v>
+        <v>21.63554078553236</v>
       </c>
       <c r="O32">
-        <v>198.5797853989933</v>
+        <v>196.3774244502621</v>
       </c>
       <c r="P32">
-        <v>206.2865578183719</v>
+        <v>208.4892170490775</v>
       </c>
       <c r="Q32">
-        <v>23530.33523264977</v>
+        <v>23269.37064694021</v>
       </c>
       <c r="R32">
-        <v>0.4604217749295739</v>
+        <v>0.0007439046380328445</v>
       </c>
     </row>
     <row r="33" spans="1:18">
@@ -2246,37 +2246,37 @@
         <v>370.6767844175679</v>
       </c>
       <c r="H33">
-        <v>205.3206703585628</v>
+        <v>202.5359534820523</v>
       </c>
       <c r="I33">
-        <v>212.003660488264</v>
+        <v>214.7883773647745</v>
       </c>
       <c r="J33">
         <v>16842.37130737565</v>
       </c>
       <c r="K33">
-        <v>26646.13920018548</v>
+        <v>26284.74376252681</v>
       </c>
       <c r="L33">
-        <v>0.0108363546376743</v>
+        <v>0.0001729756062536362</v>
       </c>
       <c r="M33">
-        <v>134.300003051758</v>
+        <v>138.240003051758</v>
       </c>
       <c r="N33">
-        <v>225.2225594880809</v>
+        <v>122.4958328476762</v>
       </c>
       <c r="O33">
-        <v>204.6518810720368</v>
+        <v>202.5361179192789</v>
       </c>
       <c r="P33">
-        <v>212.67244977479</v>
+        <v>214.7885418097816</v>
       </c>
       <c r="Q33">
-        <v>26559.34495587854</v>
+        <v>26284.76510288782</v>
       </c>
       <c r="R33">
-        <v>0.5973544683634713</v>
+        <v>0.0001686772827677555</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -2302,37 +2302,37 @@
         <v>381.9618419745027</v>
       </c>
       <c r="H34">
-        <v>211.4173281314331</v>
+        <v>208.6917732975846</v>
       </c>
       <c r="I34">
-        <v>218.3649903448552</v>
+        <v>221.0905451787038</v>
       </c>
       <c r="J34">
         <v>19898.83188489561</v>
       </c>
       <c r="K34">
-        <v>29823.2089562075</v>
+        <v>29438.73341652547</v>
       </c>
       <c r="L34">
-        <v>0.03023388880148443</v>
+        <v>0.003168324276997596</v>
       </c>
       <c r="M34">
-        <v>165.740005493164</v>
+        <v>169.680005493164</v>
       </c>
       <c r="N34">
-        <v>25.61433402967278</v>
+        <v>1.25771761094449</v>
       </c>
       <c r="O34">
-        <v>210.7220522198187</v>
+        <v>208.6919530348944</v>
       </c>
       <c r="P34">
-        <v>219.0602662564697</v>
+        <v>221.090724923887</v>
       </c>
       <c r="Q34">
-        <v>29725.13109770101</v>
+        <v>29438.75877084904</v>
       </c>
       <c r="R34">
-        <v>0.7554301712105329</v>
+        <v>0.003148122521948395</v>
       </c>
     </row>
     <row r="35" spans="1:18">
@@ -2358,37 +2358,37 @@
         <v>393.2468995314375</v>
       </c>
       <c r="H35">
-        <v>217.5125587950426</v>
+        <v>214.8448347492987</v>
       </c>
       <c r="I35">
-        <v>224.7277473107073</v>
+        <v>227.3954713564512</v>
       </c>
       <c r="J35">
         <v>23209.99751054224</v>
       </c>
       <c r="K35">
-        <v>33137.66356233606</v>
+        <v>32731.24040040583</v>
       </c>
       <c r="L35">
-        <v>0.06006773257725708</v>
+        <v>0.01044117832187113</v>
       </c>
       <c r="M35">
-        <v>56.23000335693401</v>
+        <v>60.170003356934</v>
       </c>
       <c r="N35">
-        <v>20.27760222622262</v>
+        <v>0.3172111889711278</v>
       </c>
       <c r="O35">
-        <v>216.7905106270981</v>
+        <v>214.8450297866899</v>
       </c>
       <c r="P35">
-        <v>225.4497954786518</v>
+        <v>227.3956664018123</v>
       </c>
       <c r="Q35">
-        <v>33027.66076802526</v>
+        <v>32731.27011401634</v>
       </c>
       <c r="R35">
-        <v>0.9353508079859983</v>
+        <v>0.01040135770720935</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -2414,37 +2414,37 @@
         <v>404.5319570883723</v>
       </c>
       <c r="H36">
-        <v>223.6065153626354</v>
+        <v>220.9952367278531</v>
       </c>
       <c r="I36">
-        <v>231.091778372576</v>
+        <v>233.7030570073583</v>
       </c>
       <c r="J36">
         <v>26775.86818431553</v>
       </c>
       <c r="K36">
-        <v>36589.4797416081</v>
+        <v>36162.18751109277</v>
       </c>
       <c r="L36">
-        <v>0.1008504095386824</v>
+        <v>0.02272127288545152</v>
       </c>
       <c r="M36">
-        <v>220.229995727539</v>
+        <v>224.169995727539</v>
       </c>
       <c r="N36">
-        <v>44.89973051035379</v>
+        <v>7.624686692667408</v>
       </c>
       <c r="O36">
-        <v>222.8574399322185</v>
+        <v>220.9954470653241</v>
       </c>
       <c r="P36">
-        <v>231.8408538029929</v>
+        <v>233.703267352899</v>
       </c>
       <c r="Q36">
-        <v>36466.90603108037</v>
+        <v>36162.22192931454</v>
       </c>
       <c r="R36">
-        <v>1.137731482177156</v>
+        <v>0.02265790636526348</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -2470,37 +2470,37 @@
         <v>415.8170146453072</v>
       </c>
       <c r="H37">
-        <v>229.6993309014234</v>
+        <v>227.1430766734426</v>
       </c>
       <c r="I37">
-        <v>237.4569504632496</v>
+        <v>240.0132046912304</v>
       </c>
       <c r="J37">
         <v>30596.44390621548</v>
       </c>
       <c r="K37">
-        <v>40178.63763518572</v>
+        <v>39731.50175574544</v>
       </c>
       <c r="L37">
-        <v>0.1530318888533582</v>
+        <v>0.04074402494955186</v>
       </c>
       <c r="M37">
-        <v>169.600006103516</v>
+        <v>173.540006103516</v>
       </c>
       <c r="N37">
-        <v>44.87203655611126</v>
+        <v>7.612590587965868</v>
       </c>
       <c r="O37">
-        <v>228.9229998353583</v>
+        <v>227.1433023109917</v>
       </c>
       <c r="P37">
-        <v>238.2332815293148</v>
+        <v>240.0134303369522</v>
       </c>
       <c r="Q37">
-        <v>40042.8430533471</v>
+        <v>39731.54122390273</v>
       </c>
       <c r="R37">
-        <v>1.363112222805872</v>
+        <v>0.04065298530984798</v>
       </c>
     </row>
     <row r="38" spans="1:18">
@@ -2526,37 +2526,37 @@
         <v>427.102072202242</v>
       </c>
       <c r="H38">
-        <v>235.7911214825619</v>
+        <v>233.2884502728751</v>
       </c>
       <c r="I38">
-        <v>243.8231475115727</v>
+        <v>246.3258187212595</v>
       </c>
       <c r="J38">
         <v>34671.7246762421</v>
       </c>
       <c r="K38">
-        <v>43905.12022619123</v>
+        <v>43439.11421350915</v>
       </c>
       <c r="L38">
-        <v>0.2170080539036305</v>
+        <v>0.06524630308105343</v>
       </c>
       <c r="M38">
-        <v>172.139999389648</v>
+        <v>176.079999389648</v>
       </c>
       <c r="N38">
-        <v>1.575839156800939</v>
+        <v>7.205196826829299</v>
       </c>
       <c r="O38">
-        <v>234.9873296389338</v>
+        <v>233.2886912105008</v>
       </c>
       <c r="P38">
-        <v>244.6269393552008</v>
+        <v>246.3260596671641</v>
       </c>
       <c r="Q38">
-        <v>43755.45141207546</v>
+        <v>43439.1590769262</v>
       </c>
       <c r="R38">
-        <v>1.61196814801608</v>
+        <v>0.06512327402154366</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -2582,37 +2582,37 @@
         <v>438.3871297591768</v>
       </c>
       <c r="H39">
-        <v>241.881988661942</v>
+        <v>239.4314512029183</v>
       </c>
       <c r="I39">
-        <v>250.1902679616542</v>
+        <v>252.6408054206779</v>
       </c>
       <c r="J39">
         <v>39001.71049439537</v>
       </c>
       <c r="K39">
-        <v>47768.91287062776</v>
+        <v>47284.95988589388</v>
       </c>
       <c r="L39">
-        <v>0.2931279952705457</v>
+        <v>0.0969626703527305</v>
       </c>
       <c r="M39">
-        <v>5.340000152588001</v>
+        <v>9.280000152588002</v>
       </c>
       <c r="N39">
-        <v>37.98280192078255</v>
+        <v>4.941938636762619</v>
       </c>
       <c r="O39">
-        <v>241.0505512249153</v>
+        <v>239.431707440619</v>
       </c>
       <c r="P39">
-        <v>251.0217053986809</v>
+        <v>252.6410616667668</v>
       </c>
       <c r="Q39">
-        <v>47604.71353232062</v>
+        <v>47285.0104898949</v>
       </c>
       <c r="R39">
-        <v>1.884718217724613</v>
+        <v>0.09680315716893774</v>
       </c>
     </row>
     <row r="40" spans="1:18">
@@ -2638,37 +2638,37 @@
         <v>449.6721873161116</v>
       </c>
       <c r="H40">
-        <v>247.9720215674928</v>
+        <v>245.572170917081</v>
       </c>
       <c r="I40">
-        <v>256.5582226855649</v>
+        <v>258.9580733359768</v>
       </c>
       <c r="J40">
         <v>43586.40136067531</v>
       </c>
       <c r="K40">
-        <v>51770.00291412485</v>
+        <v>51268.97753884286</v>
       </c>
       <c r="L40">
-        <v>0.3817002735670845</v>
+        <v>0.1366220840693752</v>
       </c>
       <c r="M40">
-        <v>34.729999542236</v>
+        <v>38.669999542236</v>
       </c>
       <c r="N40">
-        <v>16.27908368175363</v>
+        <v>0.00899270332286399</v>
       </c>
       <c r="O40">
-        <v>247.1127715598946</v>
+        <v>245.5724424548552</v>
       </c>
       <c r="P40">
-        <v>257.4174726931631</v>
+        <v>258.9583448822514</v>
       </c>
       <c r="Q40">
-        <v>51590.61422698132</v>
+        <v>51269.03422875197</v>
       </c>
       <c r="R40">
-        <v>2.181732749939935</v>
+        <v>0.136421423911374</v>
       </c>
     </row>
     <row r="41" spans="1:18">
@@ -2694,37 +2694,37 @@
         <v>460.9572448730464</v>
       </c>
       <c r="H41">
-        <v>254.0612986575061</v>
+        <v>251.7106984726677</v>
       </c>
       <c r="I41">
-        <v>262.9269332250132</v>
+        <v>265.2775334098516</v>
       </c>
       <c r="J41">
         <v>48425.79727508192</v>
       </c>
       <c r="K41">
-        <v>55908.37937762152</v>
+        <v>55391.10953922627</v>
       </c>
       <c r="L41">
-        <v>0.4829982898005652</v>
+        <v>0.1849450303632487</v>
       </c>
       <c r="M41">
-        <v>120.470001220703</v>
+        <v>124.410001220703</v>
       </c>
       <c r="N41">
-        <v>12.53663680945795</v>
+        <v>0.1591882746560856</v>
       </c>
       <c r="O41">
-        <v>253.1740848053336</v>
+        <v>251.7109853105141</v>
       </c>
       <c r="P41">
-        <v>263.8141470771858</v>
+        <v>265.2778202563132</v>
       </c>
       <c r="Q41">
-        <v>55713.14031957351</v>
+        <v>55391.1726603676</v>
       </c>
       <c r="R41">
-        <v>2.503339865984894</v>
+        <v>0.1846984020549281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>